<commit_message>
chore(examples): pools-example-small-3-teams uses -t 3 (3 bouts per team match)
Switch the small-3-teams example from -t 5 to -t 3 so each team match has
3 bouts (matching the team size users typically run for the small case).
CSV is unchanged — still 3 entries representing 3 teams.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pools-example-small-3-teams.xlsx
+++ b/pools-example-small-3-teams.xlsx
@@ -18,9 +18,9 @@
   </sheets>
   <definedNames>
     <definedName localSheetId="2" name="_xlnm.Print_Area">'Pool Draw'!$B$2:$F$11</definedName>
-    <definedName localSheetId="3" name="_xlnm.Print_Area">'Pool Matches'!$A$1:$H$44</definedName>
+    <definedName localSheetId="3" name="_xlnm.Print_Area">'Pool Matches'!$A$1:$H$38</definedName>
     <definedName localSheetId="6" name="_xlnm.Print_Area">'Names to Print A'!$A$1:$B$3</definedName>
-    <definedName localSheetId="4" name="_xlnm.Print_Area">'Elimination Matches'!$A$1:$H$22</definedName>
+    <definedName localSheetId="4" name="_xlnm.Print_Area">'Elimination Matches'!$A$1:$H$20</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
@@ -935,7 +935,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" s="2">
         <v>3</v>
@@ -1041,7 +1041,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="3">
@@ -1301,17 +1301,17 @@
         <f>'data'!$B$4</f>
       </c>
       <c r="B4" s="14" t="str">
-        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) ),1,0))</f>
       </c>
       <c r="C4" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) </f>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) </f>
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) </f>
       </c>
       <c r="F4" s="14" t="str">
-        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) ),1,0))</f>
+        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) ),1,0))</f>
       </c>
       <c r="G4" s="14" t="str">
         <f>'data'!$B$3</f>
@@ -1356,71 +1356,71 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="14">
-        <v>4</v>
-      </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="14">
-        <v>4</v>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="14">
-        <v>5</v>
-      </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="14">
-        <v>5</v>
+      <c r="A9" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="str">
+        <f>'data'!$B$5</f>
+      </c>
+      <c r="B10" s="14" t="str">
+        <f>IF(UPPER(D11)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C11," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F11," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D12)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C12," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F12," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D13)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-","")) ),1,0))</f>
+      </c>
+      <c r="C10" s="14" t="str">
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")) </f>
+      </c>
+      <c r="D10" s="18"/>
+      <c r="E10" s="14" t="str">
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-","")) </f>
+      </c>
+      <c r="F10" s="14" t="str">
+        <f>IF(UPPER(D11)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F11," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C11," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D12)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F12," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B12," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C12," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D13)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")) ),1,0))</f>
+      </c>
+      <c r="G10" s="14" t="str">
+        <f>'data'!$B$3</f>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="16" t="s">
-        <v>23</v>
+      <c r="A11" s="14">
+        <v>1</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="14">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="str">
-        <f>'data'!$B$5</f>
-      </c>
-      <c r="B12" s="14" t="str">
-        <f>IF(UPPER(D13)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D14)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C14," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F14," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D15)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C15," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F15," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D16)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C16," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F16," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D17)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-","")) ),1,0))</f>
-      </c>
-      <c r="C12" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")) </f>
-      </c>
+      <c r="A12" s="14">
+        <v>2</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="18"/>
-      <c r="E12" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-","")) </f>
-      </c>
-      <c r="F12" s="14" t="str">
-        <f>IF(UPPER(D13)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D14)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F14," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B14," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C14," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D15)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F15," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B15," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C15," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D16)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F16," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B16," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C16," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D17)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")) ),1,0))</f>
-      </c>
-      <c r="G12" s="14" t="str">
-        <f>'data'!$B$3</f>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="14">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="18"/>
@@ -1428,51 +1428,48 @@
       <c r="E13" s="18"/>
       <c r="F13" s="18"/>
       <c r="G13" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14">
-        <v>2</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="14">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14">
-        <v>3</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="14">
-        <v>3</v>
+      <c r="A15" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="16" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14">
-        <v>4</v>
-      </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
+      <c r="A16" s="14" t="str">
+        <f>'data'!$B$5</f>
+      </c>
+      <c r="B16" s="14" t="str">
+        <f>IF(UPPER(D17)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D18)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C18," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D19)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C19," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E19," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"0",""),"-","")) ),1,0))</f>
+      </c>
+      <c r="C16" s="14" t="str">
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C19," ",""),"0",""),"-","")) </f>
+      </c>
       <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="14">
-        <v>4</v>
+      <c r="E16" s="14" t="str">
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E19," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"0",""),"-","")) </f>
+      </c>
+      <c r="F16" s="14" t="str">
+        <f>IF(UPPER(D17)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D18)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B18," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C18," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D19)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E19," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C19," ",""),"0",""),"-","")) ),1,0))</f>
+      </c>
+      <c r="G16" s="14" t="str">
+        <f>'data'!$B$4</f>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B17" s="18"/>
       <c r="C17" s="18"/>
@@ -1480,295 +1477,220 @@
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
       <c r="G17" s="14">
-        <v>5</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14">
+        <v>2</v>
+      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="14">
+        <v>2</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="str">
+      <c r="A19" s="14">
+        <v>3</v>
+      </c>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="str">
+        <f>'data'!$B$3</f>
+      </c>
+      <c r="B23" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(F4&gt;B4,AND(F4=B4,E4&gt;C4)),1,0)),0)+IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,D11="X",D11="x",D12="X",D12="x",D13="X",D13="x",OR(D10="X",D10="x")),IF(OR(OR(D10="X",D10="x"),AND(B10=F10,C10=E10)),0,IF(OR(F10&gt;B10,AND(F10=B10,E10&gt;C10)),1,0)),0)</f>
+      </c>
+      <c r="C23" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(F4&lt;B4,AND(F4=B4,E4&lt;C4)),1,0)),0)+IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,D11="X",D11="x",D12="X",D12="x",D13="X",D13="x",OR(D10="X",D10="x")),IF(OR(OR(D10="X",D10="x"),AND(B10=F10,C10=E10)),0,IF(OR(F10&lt;B10,AND(F10=B10,E10&lt;C10)),1,0)),0)</f>
+      </c>
+      <c r="D23" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),1,0),0)+IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,D11="X",D11="x",D12="X",D12="x",D13="X",D13="x",OR(D10="X",D10="x")),IF(OR(OR(D10="X",D10="x"),AND(B10=F10,C10=E10)),1,0),0)</f>
+      </c>
+      <c r="G23" s="18" t="str">
+        <f>RANK(U23,$U$23:$U$25)+COUNTIF($U$22:U22,U23)</f>
+      </c>
+      <c r="U23" t="str">
+        <f>(B23*1000000000)-(C23*10000000)+(D23*100000)+(B28*1000)-(C28*100)+(D28*10)+(E28*1)-(F28*0.01)</f>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="str">
+        <f>'data'!$B$4</f>
+      </c>
+      <c r="B24" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(B4&gt;F4,AND(B4=F4,C4&gt;E4)),1,0)),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,D17="X",D17="x",D18="X",D18="x",D19="X",D19="x",OR(D16="X",D16="x")),IF(OR(OR(D16="X",D16="x"),AND(B16=F16,C16=E16)),0,IF(OR(F16&gt;B16,AND(F16=B16,E16&gt;C16)),1,0)),0)</f>
+      </c>
+      <c r="C24" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(B4&lt;F4,AND(B4=F4,C4&lt;E4)),1,0)),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,D17="X",D17="x",D18="X",D18="x",D19="X",D19="x",OR(D16="X",D16="x")),IF(OR(OR(D16="X",D16="x"),AND(B16=F16,C16=E16)),0,IF(OR(F16&lt;B16,AND(F16=B16,E16&lt;C16)),1,0)),0)</f>
+      </c>
+      <c r="D24" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),1,0),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,D17="X",D17="x",D18="X",D18="x",D19="X",D19="x",OR(D16="X",D16="x")),IF(OR(OR(D16="X",D16="x"),AND(B16=F16,C16=E16)),1,0),0)</f>
+      </c>
+      <c r="G24" s="18" t="str">
+        <f>RANK(U24,$U$23:$U$25)+COUNTIF($U$22:U23,U24)</f>
+      </c>
+      <c r="U24" t="str">
+        <f>(B24*1000000000)-(C24*10000000)+(D24*100000)+(B29*1000)-(C29*100)+(D29*10)+(E29*1)-(F29*0.01)</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="str">
         <f>'data'!$B$5</f>
       </c>
-      <c r="B20" s="14" t="str">
-        <f>IF(UPPER(D21)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D22)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D23)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D24)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D25)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-","")) ),1,0))</f>
-      </c>
-      <c r="C20" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")) </f>
-      </c>
-      <c r="D20" s="18"/>
-      <c r="E20" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-","")) </f>
-      </c>
-      <c r="F20" s="14" t="str">
-        <f>IF(UPPER(D21)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D22)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D23)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D24)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D25)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")) ),1,0))</f>
-      </c>
-      <c r="G20" s="14" t="str">
-        <f>'data'!$B$4</f>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14">
-        <v>1</v>
-      </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14">
-        <v>2</v>
-      </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="14">
-        <v>3</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="14">
-        <v>4</v>
-      </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="14">
-        <v>5</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="14">
-        <v>5</v>
+      <c r="B25" s="14" t="str">
+        <f>IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,D11="X",D11="x",D12="X",D12="x",D13="X",D13="x",OR(D10="X",D10="x")),IF(OR(OR(D10="X",D10="x"),AND(B10=F10,C10=E10)),0,IF(OR(B10&gt;F10,AND(B10=F10,C10&gt;E10)),1,0)),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,D17="X",D17="x",D18="X",D18="x",D19="X",D19="x",OR(D16="X",D16="x")),IF(OR(OR(D16="X",D16="x"),AND(B16=F16,C16=E16)),0,IF(OR(B16&gt;F16,AND(B16=F16,C16&gt;E16)),1,0)),0)</f>
+      </c>
+      <c r="C25" s="14" t="str">
+        <f>IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,D11="X",D11="x",D12="X",D12="x",D13="X",D13="x",OR(D10="X",D10="x")),IF(OR(OR(D10="X",D10="x"),AND(B10=F10,C10=E10)),0,IF(OR(B10&lt;F10,AND(B10=F10,C10&lt;E10)),1,0)),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,D17="X",D17="x",D18="X",D18="x",D19="X",D19="x",OR(D16="X",D16="x")),IF(OR(OR(D16="X",D16="x"),AND(B16=F16,C16=E16)),0,IF(OR(B16&lt;F16,AND(B16=F16,C16&lt;E16)),1,0)),0)</f>
+      </c>
+      <c r="D25" s="14" t="str">
+        <f>IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,D11="X",D11="x",D12="X",D12="x",D13="X",D13="x",OR(D10="X",D10="x")),IF(OR(OR(D10="X",D10="x"),AND(B10=F10,C10=E10)),1,0),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,D17="X",D17="x",D18="X",D18="x",D19="X",D19="x",OR(D16="X",D16="x")),IF(OR(OR(D16="X",D16="x"),AND(B16=F16,C16=E16)),1,0),0)</f>
+      </c>
+      <c r="G25" s="18" t="str">
+        <f>RANK(U25,$U$23:$U$25)+COUNTIF($U$22:U24,U25)</f>
+      </c>
+      <c r="U25" t="str">
+        <f>(B25*1000000000)-(C25*10000000)+(D25*100000)+(B30*1000)-(C30*100)+(D30*10)+(E30*1)-(F30*0.01)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13"/>
+      <c r="B27" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13" t="s">
-        <v>28</v>
+      <c r="A28" s="14" t="str">
+        <f>'data'!$B$3</f>
+      </c>
+      <c r="B28" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X"),F4,0)+IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,OR(D10="X",D10="x"),UPPER(D11)="X",UPPER(D12)="X",UPPER(D13)="X"),F10,0)</f>
+      </c>
+      <c r="C28" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X"),B4,0)+IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,OR(D10="X",D10="x"),UPPER(D11)="X",UPPER(D12)="X",UPPER(D13)="X"),B10,0)</f>
+      </c>
+      <c r="D28" s="14" t="str">
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X"),(IF(OR(D5="X",D5="x",AND(COUNTA(B5,C5,E5,F5)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-",""))))),1,0)+IF(OR(D6="X",D6="x",AND(COUNTA(B6,C6,E6,F6)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-",""))))),1,0)+IF(OR(D7="X",D7="x",AND(COUNTA(B7,C7,E7,F7)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-",""))))),1,0)),0)+IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,OR(D10="X",D10="x"),UPPER(D11)="X",UPPER(D12)="X",UPPER(D13)="X"),(IF(OR(D11="X",D11="x",AND(COUNTA(B11,C11,E11,F11)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C11," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E11," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F11," ",""),"0",""),"-",""))))),1,0)+IF(OR(D12="X",D12="x",AND(COUNTA(B12,C12,E12,F12)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B12," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C12," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E12," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F12," ",""),"0",""),"-",""))))),1,0)+IF(OR(D13="X",D13="x",AND(COUNTA(B13,C13,E13,F13)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-",""))))),1,0)),0)</f>
+      </c>
+      <c r="E28" s="14" t="str">
+        <f>E4+E10</f>
+      </c>
+      <c r="F28" s="14" t="str">
+        <f>C4+C10</f>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="str">
-        <f>'data'!$B$3</f>
+        <f>'data'!$B$4</f>
       </c>
       <c r="B29" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",D8="X",D8="x",D9="X",D9="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(F4&gt;B4,AND(F4=B4,E4&gt;C4)),1,0)),0)+IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,D13="X",D13="x",D14="X",D14="x",D15="X",D15="x",D16="X",D16="x",D17="X",D17="x",OR(D12="X",D12="x")),IF(OR(OR(D12="X",D12="x"),AND(B12=F12,C12=E12)),0,IF(OR(F12&gt;B12,AND(F12=B12,E12&gt;C12)),1,0)),0)</f>
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X"),B4,0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,OR(D16="X",D16="x"),UPPER(D17)="X",UPPER(D18)="X",UPPER(D19)="X"),F16,0)</f>
       </c>
       <c r="C29" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",D8="X",D8="x",D9="X",D9="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(F4&lt;B4,AND(F4=B4,E4&lt;C4)),1,0)),0)+IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,D13="X",D13="x",D14="X",D14="x",D15="X",D15="x",D16="X",D16="x",D17="X",D17="x",OR(D12="X",D12="x")),IF(OR(OR(D12="X",D12="x"),AND(B12=F12,C12=E12)),0,IF(OR(F12&lt;B12,AND(F12=B12,E12&lt;C12)),1,0)),0)</f>
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X"),F4,0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,OR(D16="X",D16="x"),UPPER(D17)="X",UPPER(D18)="X",UPPER(D19)="X"),B16,0)</f>
       </c>
       <c r="D29" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",D8="X",D8="x",D9="X",D9="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),1,0),0)+IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,D13="X",D13="x",D14="X",D14="x",D15="X",D15="x",D16="X",D16="x",D17="X",D17="x",OR(D12="X",D12="x")),IF(OR(OR(D12="X",D12="x"),AND(B12=F12,C12=E12)),1,0),0)</f>
-      </c>
-      <c r="G29" s="18" t="str">
-        <f>RANK(U29,$U$29:$U$31)+COUNTIF($U$28:U28,U29)</f>
-      </c>
-      <c r="U29" t="str">
-        <f>(B29*1000000000)-(C29*10000000)+(D29*100000)+(B34*1000)-(C34*100)+(D34*10)+(E34*1)-(F34*0.01)</f>
+        <f>IF(OR(COUNTA(B5:C7,E5:F7)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X"),(IF(OR(D5="X",D5="x",AND(COUNTA(B5,C5,E5,F5)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-",""))))),1,0)+IF(OR(D6="X",D6="x",AND(COUNTA(B6,C6,E6,F6)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-",""))))),1,0)+IF(OR(D7="X",D7="x",AND(COUNTA(B7,C7,E7,F7)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-",""))))),1,0)),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,OR(D16="X",D16="x"),UPPER(D17)="X",UPPER(D18)="X",UPPER(D19)="X"),(IF(OR(D17="X",D17="x",AND(COUNTA(B17,C17,E17,F17)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-",""))))),1,0)+IF(OR(D18="X",D18="x",AND(COUNTA(B18,C18,E18,F18)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B18," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C18," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E18," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"0",""),"-",""))))),1,0)+IF(OR(D19="X",D19="x",AND(COUNTA(B19,C19,E19,F19)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C19," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E19," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"0",""),"-",""))))),1,0)),0)</f>
+      </c>
+      <c r="E29" s="14" t="str">
+        <f>C4+E16</f>
+      </c>
+      <c r="F29" s="14" t="str">
+        <f>E4+C16</f>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="str">
-        <f>'data'!$B$4</f>
+        <f>'data'!$B$5</f>
       </c>
       <c r="B30" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",D8="X",D8="x",D9="X",D9="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(B4&gt;F4,AND(B4=F4,C4&gt;E4)),1,0)),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,D21="X",D21="x",D22="X",D22="x",D23="X",D23="x",D24="X",D24="x",D25="X",D25="x",OR(D20="X",D20="x")),IF(OR(OR(D20="X",D20="x"),AND(B20=F20,C20=E20)),0,IF(OR(F20&gt;B20,AND(F20=B20,E20&gt;C20)),1,0)),0)</f>
+        <f>IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,OR(D10="X",D10="x"),UPPER(D11)="X",UPPER(D12)="X",UPPER(D13)="X"),B10,0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,OR(D16="X",D16="x"),UPPER(D17)="X",UPPER(D18)="X",UPPER(D19)="X"),B16,0)</f>
       </c>
       <c r="C30" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",D8="X",D8="x",D9="X",D9="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),0,IF(OR(B4&lt;F4,AND(B4=F4,C4&lt;E4)),1,0)),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,D21="X",D21="x",D22="X",D22="x",D23="X",D23="x",D24="X",D24="x",D25="X",D25="x",OR(D20="X",D20="x")),IF(OR(OR(D20="X",D20="x"),AND(B20=F20,C20=E20)),0,IF(OR(F20&lt;B20,AND(F20=B20,E20&lt;C20)),1,0)),0)</f>
+        <f>IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,OR(D10="X",D10="x"),UPPER(D11)="X",UPPER(D12)="X",UPPER(D13)="X"),F10,0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,OR(D16="X",D16="x"),UPPER(D17)="X",UPPER(D18)="X",UPPER(D19)="X"),F16,0)</f>
       </c>
       <c r="D30" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,D5="X",D5="x",D6="X",D6="x",D7="X",D7="x",D8="X",D8="x",D9="X",D9="x",OR(D4="X",D4="x")),IF(OR(OR(D4="X",D4="x"),AND(B4=F4,C4=E4)),1,0),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,D21="X",D21="x",D22="X",D22="x",D23="X",D23="x",D24="X",D24="x",D25="X",D25="x",OR(D20="X",D20="x")),IF(OR(OR(D20="X",D20="x"),AND(B20=F20,C20=E20)),1,0),0)</f>
-      </c>
-      <c r="G30" s="18" t="str">
-        <f>RANK(U30,$U$29:$U$31)+COUNTIF($U$28:U29,U30)</f>
-      </c>
-      <c r="U30" t="str">
-        <f>(B30*1000000000)-(C30*10000000)+(D30*100000)+(B35*1000)-(C35*100)+(D35*10)+(E35*1)-(F35*0.01)</f>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="14" t="str">
-        <f>'data'!$B$5</f>
-      </c>
-      <c r="B31" s="14" t="str">
-        <f>IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,D13="X",D13="x",D14="X",D14="x",D15="X",D15="x",D16="X",D16="x",D17="X",D17="x",OR(D12="X",D12="x")),IF(OR(OR(D12="X",D12="x"),AND(B12=F12,C12=E12)),0,IF(OR(B12&gt;F12,AND(B12=F12,C12&gt;E12)),1,0)),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,D21="X",D21="x",D22="X",D22="x",D23="X",D23="x",D24="X",D24="x",D25="X",D25="x",OR(D20="X",D20="x")),IF(OR(OR(D20="X",D20="x"),AND(B20=F20,C20=E20)),0,IF(OR(B20&gt;F20,AND(B20=F20,C20&gt;E20)),1,0)),0)</f>
-      </c>
-      <c r="C31" s="14" t="str">
-        <f>IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,D13="X",D13="x",D14="X",D14="x",D15="X",D15="x",D16="X",D16="x",D17="X",D17="x",OR(D12="X",D12="x")),IF(OR(OR(D12="X",D12="x"),AND(B12=F12,C12=E12)),0,IF(OR(B12&lt;F12,AND(B12=F12,C12&lt;E12)),1,0)),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,D21="X",D21="x",D22="X",D22="x",D23="X",D23="x",D24="X",D24="x",D25="X",D25="x",OR(D20="X",D20="x")),IF(OR(OR(D20="X",D20="x"),AND(B20=F20,C20=E20)),0,IF(OR(B20&lt;F20,AND(B20=F20,C20&lt;E20)),1,0)),0)</f>
-      </c>
-      <c r="D31" s="14" t="str">
-        <f>IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,D13="X",D13="x",D14="X",D14="x",D15="X",D15="x",D16="X",D16="x",D17="X",D17="x",OR(D12="X",D12="x")),IF(OR(OR(D12="X",D12="x"),AND(B12=F12,C12=E12)),1,0),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,D21="X",D21="x",D22="X",D22="x",D23="X",D23="x",D24="X",D24="x",D25="X",D25="x",OR(D20="X",D20="x")),IF(OR(OR(D20="X",D20="x"),AND(B20=F20,C20=E20)),1,0),0)</f>
-      </c>
-      <c r="G31" s="18" t="str">
-        <f>RANK(U31,$U$29:$U$31)+COUNTIF($U$28:U30,U31)</f>
-      </c>
-      <c r="U31" t="str">
-        <f>(B31*1000000000)-(C31*10000000)+(D31*100000)+(B36*1000)-(C36*100)+(D36*10)+(E36*1)-(F36*0.01)</f>
+        <f>IF(OR(COUNTA(B11:C13,E11:F13)&gt;0,OR(D10="X",D10="x"),UPPER(D11)="X",UPPER(D12)="X",UPPER(D13)="X"),(IF(OR(D11="X",D11="x",AND(COUNTA(B11,C11,E11,F11)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C11," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E11," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F11," ",""),"0",""),"-",""))))),1,0)+IF(OR(D12="X",D12="x",AND(COUNTA(B12,C12,E12,F12)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B12," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C12," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E12," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F12," ",""),"0",""),"-",""))))),1,0)+IF(OR(D13="X",D13="x",AND(COUNTA(B13,C13,E13,F13)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-",""))))),1,0)),0)+IF(OR(COUNTA(B17:C19,E17:F19)&gt;0,OR(D16="X",D16="x"),UPPER(D17)="X",UPPER(D18)="X",UPPER(D19)="X"),(IF(OR(D17="X",D17="x",AND(COUNTA(B17,C17,E17,F17)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-",""))))),1,0)+IF(OR(D18="X",D18="x",AND(COUNTA(B18,C18,E18,F18)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B18," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C18," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E18," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"0",""),"-",""))))),1,0)+IF(OR(D19="X",D19="x",AND(COUNTA(B19,C19,E19,F19)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C19," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E19," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"0",""),"-",""))))),1,0)),0)</f>
+      </c>
+      <c r="E30" s="14" t="str">
+        <f>C10+C16</f>
+      </c>
+      <c r="F30" s="14" t="str">
+        <f>E10+E16</f>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F33" s="13" t="s">
-        <v>33</v>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="str">
-        <f>'data'!$B$3</f>
-      </c>
-      <c r="B34" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X",UPPER(D8)="X",UPPER(D9)="X"),F4,0)+IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,OR(D12="X",D12="x"),UPPER(D13)="X",UPPER(D14)="X",UPPER(D15)="X",UPPER(D16)="X",UPPER(D17)="X"),F12,0)</f>
-      </c>
-      <c r="C34" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X",UPPER(D8)="X",UPPER(D9)="X"),B4,0)+IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,OR(D12="X",D12="x"),UPPER(D13)="X",UPPER(D14)="X",UPPER(D15)="X",UPPER(D16)="X",UPPER(D17)="X"),B12,0)</f>
-      </c>
-      <c r="D34" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X",UPPER(D8)="X",UPPER(D9)="X"),(IF(OR(D5="X",D5="x",AND(COUNTA(B5,C5,E5,F5)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-",""))))),1,0)+IF(OR(D6="X",D6="x",AND(COUNTA(B6,C6,E6,F6)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-",""))))),1,0)+IF(OR(D7="X",D7="x",AND(COUNTA(B7,C7,E7,F7)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-",""))))),1,0)+IF(OR(D8="X",D8="x",AND(COUNTA(B8,C8,E8,F8)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-",""))))),1,0)+IF(OR(D9="X",D9="x",AND(COUNTA(B9,C9,E9,F9)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-",""))))),1,0)),0)+IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,OR(D12="X",D12="x"),UPPER(D13)="X",UPPER(D14)="X",UPPER(D15)="X",UPPER(D16)="X",UPPER(D17)="X"),(IF(OR(D13="X",D13="x",AND(COUNTA(B13,C13,E13,F13)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-",""))))),1,0)+IF(OR(D14="X",D14="x",AND(COUNTA(B14,C14,E14,F14)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B14," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C14," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E14," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F14," ",""),"0",""),"-",""))))),1,0)+IF(OR(D15="X",D15="x",AND(COUNTA(B15,C15,E15,F15)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B15," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C15," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E15," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F15," ",""),"0",""),"-",""))))),1,0)+IF(OR(D16="X",D16="x",AND(COUNTA(B16,C16,E16,F16)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B16," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C16," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E16," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F16," ",""),"0",""),"-",""))))),1,0)+IF(OR(D17="X",D17="x",AND(COUNTA(B17,C17,E17,F17)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-",""))))),1,0)),0)</f>
-      </c>
-      <c r="E34" s="14" t="str">
-        <f>E4+E12</f>
-      </c>
-      <c r="F34" s="14" t="str">
-        <f>C4+C12</f>
+      <c r="F34" t="s">
+        <v>35</v>
+      </c>
+      <c r="G34" s="19" t="str">
+        <f>IFERROR(INDEX($A$23:$A$30, MATCH(1, $G$23:$G$30, 0)), "-")</f>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="str">
-        <f>'data'!$B$4</f>
-      </c>
-      <c r="B35" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X",UPPER(D8)="X",UPPER(D9)="X"),B4,0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,OR(D20="X",D20="x"),UPPER(D21)="X",UPPER(D22)="X",UPPER(D23)="X",UPPER(D24)="X",UPPER(D25)="X"),F20,0)</f>
-      </c>
-      <c r="C35" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X",UPPER(D8)="X",UPPER(D9)="X"),F4,0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,OR(D20="X",D20="x"),UPPER(D21)="X",UPPER(D22)="X",UPPER(D23)="X",UPPER(D24)="X",UPPER(D25)="X"),B20,0)</f>
-      </c>
-      <c r="D35" s="14" t="str">
-        <f>IF(OR(COUNTA(B5:C9,E5:F9)&gt;0,OR(D4="X",D4="x"),UPPER(D5)="X",UPPER(D6)="X",UPPER(D7)="X",UPPER(D8)="X",UPPER(D9)="X"),(IF(OR(D5="X",D5="x",AND(COUNTA(B5,C5,E5,F5)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-",""))))),1,0)+IF(OR(D6="X",D6="x",AND(COUNTA(B6,C6,E6,F6)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-",""))))),1,0)+IF(OR(D7="X",D7="x",AND(COUNTA(B7,C7,E7,F7)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-",""))))),1,0)+IF(OR(D8="X",D8="x",AND(COUNTA(B8,C8,E8,F8)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-",""))))),1,0)+IF(OR(D9="X",D9="x",AND(COUNTA(B9,C9,E9,F9)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-",""))))),1,0)),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,OR(D20="X",D20="x"),UPPER(D21)="X",UPPER(D22)="X",UPPER(D23)="X",UPPER(D24)="X",UPPER(D25)="X"),(IF(OR(D21="X",D21="x",AND(COUNTA(B21,C21,E21,F21)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-",""))))),1,0)+IF(OR(D22="X",D22="x",AND(COUNTA(B22,C22,E22,F22)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-",""))))),1,0)+IF(OR(D23="X",D23="x",AND(COUNTA(B23,C23,E23,F23)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-",""))))),1,0)+IF(OR(D24="X",D24="x",AND(COUNTA(B24,C24,E24,F24)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-",""))))),1,0)+IF(OR(D25="X",D25="x",AND(COUNTA(B25,C25,E25,F25)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-",""))))),1,0)),0)</f>
-      </c>
-      <c r="E35" s="14" t="str">
-        <f>C4+E20</f>
-      </c>
-      <c r="F35" s="14" t="str">
-        <f>E4+C20</f>
+      <c r="F35" t="s">
+        <v>36</v>
+      </c>
+      <c r="G35" s="19" t="str">
+        <f>IFERROR(INDEX($A$23:$A$30, MATCH(2, $G$23:$G$30, 0)), "-")</f>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="str">
-        <f>'data'!$B$5</f>
-      </c>
-      <c r="B36" s="14" t="str">
-        <f>IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,OR(D12="X",D12="x"),UPPER(D13)="X",UPPER(D14)="X",UPPER(D15)="X",UPPER(D16)="X",UPPER(D17)="X"),B12,0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,OR(D20="X",D20="x"),UPPER(D21)="X",UPPER(D22)="X",UPPER(D23)="X",UPPER(D24)="X",UPPER(D25)="X"),B20,0)</f>
-      </c>
-      <c r="C36" s="14" t="str">
-        <f>IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,OR(D12="X",D12="x"),UPPER(D13)="X",UPPER(D14)="X",UPPER(D15)="X",UPPER(D16)="X",UPPER(D17)="X"),F12,0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,OR(D20="X",D20="x"),UPPER(D21)="X",UPPER(D22)="X",UPPER(D23)="X",UPPER(D24)="X",UPPER(D25)="X"),F20,0)</f>
-      </c>
-      <c r="D36" s="14" t="str">
-        <f>IF(OR(COUNTA(B13:C17,E13:F17)&gt;0,OR(D12="X",D12="x"),UPPER(D13)="X",UPPER(D14)="X",UPPER(D15)="X",UPPER(D16)="X",UPPER(D17)="X"),(IF(OR(D13="X",D13="x",AND(COUNTA(B13,C13,E13,F13)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C13," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E13," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F13," ",""),"0",""),"-",""))))),1,0)+IF(OR(D14="X",D14="x",AND(COUNTA(B14,C14,E14,F14)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B14," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C14," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E14," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F14," ",""),"0",""),"-",""))))),1,0)+IF(OR(D15="X",D15="x",AND(COUNTA(B15,C15,E15,F15)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B15," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C15," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E15," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F15," ",""),"0",""),"-",""))))),1,0)+IF(OR(D16="X",D16="x",AND(COUNTA(B16,C16,E16,F16)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B16," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C16," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E16," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F16," ",""),"0",""),"-",""))))),1,0)+IF(OR(D17="X",D17="x",AND(COUNTA(B17,C17,E17,F17)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C17," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E17," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F17," ",""),"0",""),"-",""))))),1,0)),0)+IF(OR(COUNTA(B21:C25,E21:F25)&gt;0,OR(D20="X",D20="x"),UPPER(D21)="X",UPPER(D22)="X",UPPER(D23)="X",UPPER(D24)="X",UPPER(D25)="X"),(IF(OR(D21="X",D21="x",AND(COUNTA(B21,C21,E21,F21)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C21," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E21," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"0",""),"-",""))))),1,0)+IF(OR(D22="X",D22="x",AND(COUNTA(B22,C22,E22,F22)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C22," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E22," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"0",""),"-",""))))),1,0)+IF(OR(D23="X",D23="x",AND(COUNTA(B23,C23,E23,F23)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C23," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E23," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F23," ",""),"0",""),"-",""))))),1,0)+IF(OR(D24="X",D24="x",AND(COUNTA(B24,C24,E24,F24)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C24," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E24," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F24," ",""),"0",""),"-",""))))),1,0)+IF(OR(D25="X",D25="x",AND(COUNTA(B25,C25,E25,F25)&gt;0,(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C25," ",""),"0",""),"-","")))=(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E25," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F25," ",""),"0",""),"-",""))))),1,0)),0)</f>
-      </c>
-      <c r="E36" s="14" t="str">
-        <f>C12+C20</f>
-      </c>
-      <c r="F36" s="14" t="str">
-        <f>E12+E20</f>
-      </c>
-    </row>
-    <row r="39">
-      <c r="F39" s="13"/>
-      <c r="G39" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="F40" t="s">
-        <v>35</v>
-      </c>
-      <c r="G40" s="19" t="str">
-        <f>IFERROR(INDEX($A$29:$A$36, MATCH(1, $G$29:$G$36, 0)), "-")</f>
-      </c>
-    </row>
-    <row r="41">
-      <c r="F41" t="s">
-        <v>36</v>
-      </c>
-      <c r="G41" s="19" t="str">
-        <f>IFERROR(INDEX($A$29:$A$36, MATCH(2, $G$29:$G$36, 0)), "-")</f>
-      </c>
-    </row>
-    <row r="42">
-      <c r="F42" t="s">
+      <c r="F36" t="s">
         <v>37</v>
       </c>
-      <c r="G42" s="19" t="str">
-        <f>IFERROR(INDEX($A$29:$A$36, MATCH(3, $G$29:$G$36, 0)), "-")</f>
+      <c r="G36" s="19" t="str">
+        <f>IFERROR(INDEX($A$23:$A$30, MATCH(3, $G$23:$G$30, 0)), "-")</f>
       </c>
     </row>
   </sheetData>
@@ -1835,7 +1757,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="str">
-        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G41)</f>
+        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G35)</f>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -1843,7 +1765,7 @@
       <c r="E4" s="14"/>
       <c r="F4" s="14"/>
       <c r="G4" s="14" t="str">
-        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G40)</f>
+        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G34)</f>
       </c>
     </row>
     <row r="5">
@@ -1885,85 +1807,59 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="14">
-        <v>4</v>
-      </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="14">
-        <v>4</v>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="14">
-        <v>5</v>
-      </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="str">
-        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G41)</f>
-      </c>
-      <c r="B11" s="14" t="s">
+      <c r="A9" s="14" t="str">
+        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G35)</f>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C9" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14" t="s">
+      <c r="D9" s="14"/>
+      <c r="E9" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F9" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="14" t="str">
-        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G40)</f>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="s">
+      <c r="G9" s="14" t="str">
+        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G34)</f>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="14" t="str">
-        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) ),1,0))</f>
-      </c>
-      <c r="C12" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) </f>
-      </c>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14" t="str">
-        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) </f>
-      </c>
-      <c r="F12" s="14" t="str">
-        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D8)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F8," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C8," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D9)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F9," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C9," ",""),"0",""),"-","")) ),1,0))</f>
-      </c>
-      <c r="G12" s="14" t="s">
+      <c r="B10" s="14" t="str">
+        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) ),1,0))</f>
+      </c>
+      <c r="C10" s="14" t="str">
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) </f>
+      </c>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14" t="str">
+        <f>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) </f>
+      </c>
+      <c r="F10" s="14" t="str">
+        <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")) ),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")) )&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-","")) +LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")) ),1,0))</f>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15">
-      <c r="F15" t="s">
+    <row r="13">
+      <c r="F13" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="19"/>
-    </row>
-    <row r="16">
-      <c r="F16" t="s">
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14">
+      <c r="F14" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="19"/>
+      <c r="G14" s="19"/>
     </row>
   </sheetData>
   <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="true" formatColumns="true" formatRows="true" insertColumns="true" insertRows="true" insertHyperlinks="true" deleteColumns="true" deleteRows="true" selectLockedCells="false" sort="true" autoFilter="true" pivotTables="true" selectUnlockedCells="false"/>
@@ -2015,7 +1911,7 @@
         <f>"1. " &amp; data!$B$3</f>
       </c>
       <c r="C5" s="23" t="str">
-        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G40)</f>
+        <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G34)</f>
       </c>
     </row>
     <row r="6">
@@ -2032,7 +1928,7 @@
         <f>"3. " &amp; data!$B$5</f>
       </c>
       <c r="C7" s="23" t="str">
-        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G41)</f>
+        <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G35)</f>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="20"/>

</xml_diff>

<commit_message>
fix(bc-drwx): give the 3-teams mock roster three distinct teams and dojos
test-data/mock_data_small_3_teams.csv put all three rows in "Team Alpha"
with individual person names (Aiko/Bunta/Chiyo Tanaka), which reads as
three PEOPLE from one dojo rather than the three separate TEAMS the
filename and the Makefile's -t 3 (team-matches) invocation intend. Each row
is now one team, with its own name and its own distinct dojo (Team
Alpha/Sakura Dojo, Team Bravo/Tora Dojo, Team Charlie/Kaze Dojo).
Regenerated pools-example-small-3-teams.xlsx via `make examples`; every
other example workbook came out byte-identical (deterministic generation),
confirming this was the only file the change touched.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pools-example-small-3-teams.xlsx
+++ b/pools-example-small-3-teams.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Number of pools</t>
   </si>
@@ -78,16 +78,22 @@
     <t>Pool A</t>
   </si>
   <si>
-    <t>Aiko Tanaka</t>
-  </si>
-  <si>
     <t>Team Alpha</t>
   </si>
   <si>
-    <t>Bunta Tanaka</t>
-  </si>
-  <si>
-    <t>Chiyo Tanaka</t>
+    <t>Sakura Dojo</t>
+  </si>
+  <si>
+    <t>Team Bravo</t>
+  </si>
+  <si>
+    <t>Tora Dojo</t>
+  </si>
+  <si>
+    <t>Team Charlie</t>
+  </si>
+  <si>
+    <t>Kaze Dojo</t>
   </si>
   <si>
     <t>Shiaijo A</t>
@@ -823,7 +829,7 @@
         <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -831,10 +837,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -852,32 +858,32 @@
   <sheetData>
     <row r="1" ht="409" customHeight="true">
       <c r="A1" s="30" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" ht="409" customHeight="true">
       <c r="A2" s="30" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" ht="409" customHeight="true">
       <c r="A3" s="30" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" ht="409" customHeight="true">
       <c r="A4" s="30" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" ht="409" customHeight="true">
       <c r="A5" s="30" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" ht="409" customHeight="true">
       <c r="A6" s="30" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1093,7 +1099,7 @@
     </row>
     <row r="13">
       <c r="E13" s="13" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
@@ -1104,7 +1110,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -1114,7 +1120,7 @@
     </row>
     <row r="15">
       <c r="E15" s="32" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -1124,7 +1130,7 @@
     </row>
     <row r="16">
       <c r="E16" s="32" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -1134,7 +1140,7 @@
     </row>
     <row r="17">
       <c r="E17" s="32" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F17" s="32"/>
       <c r="G17" s="32"/>
@@ -1144,7 +1150,7 @@
     </row>
     <row r="18">
       <c r="E18" s="13" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F18" s="13"/>
       <c r="G18" s="13"/>
@@ -1154,7 +1160,7 @@
     </row>
     <row r="19">
       <c r="E19" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
@@ -1262,7 +1268,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -1284,17 +1290,17 @@
     </row>
     <row r="3">
       <c r="A3" s="17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
       <c r="D3" s="14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="14"/>
       <c r="G3" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -1359,17 +1365,17 @@
     </row>
     <row r="9">
       <c r="A9" s="17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
       <c r="D9" s="14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -1434,17 +1440,17 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E15" s="14"/>
       <c r="F15" s="14"/>
       <c r="G15" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -1509,21 +1515,21 @@
     </row>
     <row r="22">
       <c r="A22" s="13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E22" s="13"/>
       <c r="F22" s="13"/>
       <c r="G22" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
@@ -1589,19 +1595,19 @@
     <row r="27">
       <c r="A27" s="13"/>
       <c r="B27" s="13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28">
@@ -1667,12 +1673,12 @@
     <row r="33">
       <c r="F33" s="13"/>
       <c r="G33" s="13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34">
       <c r="F34" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G34" s="19" t="str">
         <f>IFERROR(INDEX($A$23:$A$30, MATCH(1, $G$23:$G$30, 0)), "-")</f>
@@ -1680,7 +1686,7 @@
     </row>
     <row r="35">
       <c r="F35" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G35" s="19" t="str">
         <f>IFERROR(INDEX($A$23:$A$30, MATCH(2, $G$23:$G$30, 0)), "-")</f>
@@ -1688,7 +1694,7 @@
     </row>
     <row r="36">
       <c r="F36" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G36" s="19" t="str">
         <f>IFERROR(INDEX($A$23:$A$30, MATCH(3, $G$23:$G$30, 0)), "-")</f>
@@ -1725,7 +1731,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -1736,7 +1742,7 @@
     </row>
     <row r="2">
       <c r="A2" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -1747,13 +1753,13 @@
     </row>
     <row r="3">
       <c r="A3" s="17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -1813,17 +1819,17 @@
         <f>CONCATENATE("Pool A-2nd ",'Pool Matches'!G35)</f>
       </c>
       <c r="B9" s="14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9" s="14" t="str">
         <f>CONCATENATE("Pool A-1st ",'Pool Matches'!G34)</f>
@@ -1831,7 +1837,7 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B10" s="14" t="str">
         <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-",""))),1,0))</f>
@@ -1847,18 +1853,18 @@
         <f>IF(UPPER(D5)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C5," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D6)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F6," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C6," ",""),"0",""),"-",""))),1,0))+IF(UPPER(D7)="X",0,IF((LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(E7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F7," ",""),"0",""),"-","")))&gt;(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7," ",""),"0",""),"-",""))+LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(C7," ",""),"0",""),"-",""))),1,0))</f>
       </c>
       <c r="G10" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13">
       <c r="F13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G13" s="19"/>
     </row>
     <row r="14">
       <c r="F14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G14" s="19"/>
     </row>
@@ -1951,7 +1957,7 @@
   <sheetData>
     <row r="1" ht="270" customHeight="true">
       <c r="A1" s="28" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B1" s="29" t="str">
         <f>'data'!$B$3</f>
@@ -1959,7 +1965,7 @@
     </row>
     <row r="2" ht="270" customHeight="true">
       <c r="A2" s="28" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B2" s="29" t="str">
         <f>'data'!$B$4</f>
@@ -1967,7 +1973,7 @@
     </row>
     <row r="3" ht="270" customHeight="true">
       <c r="A3" s="28" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B3" s="29" t="str">
         <f>'data'!$B$5</f>

</xml_diff>